<commit_message>
Register: show NOT FOR USE status (204-003)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-204.xlsx
+++ b/docs/Register-SWI-204.xlsx
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +45,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,7 +95,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -803,9 +811,9 @@
           <t>Tidak ada padanan</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Final (isi tanpa tambahan)</t>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOR USE (menunggu input)</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -1920,46 +1928,46 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>No. dokumen</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Jenis</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Isi catatan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Tidak ada draft, catatan, atau open items di seri ini.</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-003</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Particle Size Distribution by Laser Sizer</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the named input arrives: a laser particle size analyser has not been purchased (no laser sizer in ILS quotation Q0023979). The method, frequency and equipment are written when the instrument is resolved.</t>
         </is>
       </c>
     </row>
@@ -1982,49 +1990,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Register seri 204 Physical Testwork (16 dokumen dalam format Heritage).</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Data dibaca langsung dari Part 1 dan Part 2 tiap dokumen (judul, tanggal, owner, JSEA ID, area, frekuensi).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Klasifikasi dan padanan Martabe diambil dari docs/Matriks-Rujukan-Martabe.xlsx dan docs/Tabel-SWI-vs-Martabe.xlsx, ditimpa oleh keputusan review bila ada. Format Heritage tidak memuat kolom klasifikasi, jadi klasifikasi hanya ada di register.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Jumlah step dan halaman dihitung dari render dokumen (LibreOffice); halaman bisa sedikit berbeda di Microsoft Word.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Status isi: Final = tanpa tambahan Martabe terbuka; DRAFT FOR REVIEW = ada tambahan Martabe yang menunggu JSEA; Catatan = ada catatan yang perlu ditindaklanjuti.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Sheet "Draft dan open items" memuat paragraf draft, catatan, temuan safety-critical, dan open items di Description of work.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Referensi register: HM-MMM-WHS-REG-XXX-R00-SWI-SWMS, tab SWI-MET.</t>
         </is>

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-204-006, 008, 010 to Heritage per Martabe decisions; 204 series complete
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-204.xlsx
+++ b/docs/Register-SWI-204.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keterangan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 204'!$A$1:$Q$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 204'!$A$1:$Q$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,7 +103,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -469,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -996,17 +1004,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>204-007</t>
+          <t>204-006</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-007</t>
+          <t>SWI-PRO-MET-204-006</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Total Suspended Solids Determination</t>
+          <t>Moisture Content Determination</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1021,7 +1029,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-007</t>
+          <t>JSEA-PRO-MET-204-006</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1046,7 +1054,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Per the sampling schedule; each shift on thickener overflow.</t>
+          <t>Every solid sample requiring a dry mass.</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
@@ -1057,7 +1065,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
+          <t>A&amp;D MS-70 Moisture Analyzer Calibration - tidak dipakai (Mt. Morgan tidak punya moisture analyser)</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
@@ -1072,24 +1080,24 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-007-Total-Suspended-Solids-Determination-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-006-Moisture-Content-Determination-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>204-009</t>
+          <t>204-007</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-009</t>
+          <t>SWI-PRO-MET-204-007</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Static and Dynamic Settling Test</t>
+          <t>Total Suspended Solids Determination</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1104,7 +1112,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-009</t>
+          <t>JSEA-PRO-MET-204-007</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1129,7 +1137,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>On each new ore type, and whenever thickener performance changes.</t>
+          <t>Per the sampling schedule; each shift on thickener overflow.</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
@@ -1155,24 +1163,24 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-009-Static-and-Dynamic-Settling-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-007-Total-Suspended-Solids-Determination-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>204-011</t>
+          <t>204-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-011</t>
+          <t>SWI-PRO-MET-204-008</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Filter Press Simulation and Cake Filtration Test</t>
+          <t>Slurry Viscosity and Rheology Test</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1187,7 +1195,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-011</t>
+          <t>JSEA-PRO-MET-204-008</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1212,23 +1220,23 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>On each new ore type and whenever plant cake moisture moves.</t>
+          <t>On each new ore type, and whenever pumping or mixing behaviour changes.</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
-        </is>
-      </c>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
-          <t>Final (isi tanpa tambahan)</t>
+          <t>Brookfield DV2TLV Viscometer dan Marsh Funnel - cara Martabe dipakai dengan alat yang sama</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1238,24 +1246,24 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-011-Filter-Press-Simulation-and-Cake-Filtration-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-008-Slurry-Viscosity-and-Rheology-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>204-012</t>
+          <t>204-009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-012</t>
+          <t>SWI-PRO-MET-204-009</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Bond Ball Mill Work Index Test</t>
+          <t>Static and Dynamic Settling Test</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1270,7 +1278,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-012</t>
+          <t>JSEA-PRO-MET-204-009</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1295,7 +1303,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>On each new ore type or ore blend.</t>
+          <t>On each new ore type, and whenever thickener performance changes.</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
@@ -1321,24 +1329,24 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-012-Bond-Ball-Mill-Work-Index-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-009-Static-and-Dynamic-Settling-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>204-013</t>
+          <t>204-010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-013</t>
+          <t>SWI-PRO-MET-204-010</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Grind Establishment Test</t>
+          <t>Flocculant Screening and Dose Optimisation Test</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1353,7 +1361,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-013</t>
+          <t>JSEA-PRO-MET-204-010</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1378,23 +1386,23 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>On each new ore type, and when a change to the grind target is proposed.</t>
+          <t>On each new ore type and when a flocculant change is proposed.</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t>Final (isi tanpa tambahan)</t>
+          <t>Settling Test Strength Variance; Effective Treatment Dosage; Flocculant Testwork on Tailing Using Sieve - Step 4-8</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1404,24 +1412,24 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-013-Grind-Establishment-Test-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-010-Flocculant-Screening-and-Dose-Optimisation-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>204-014</t>
+          <t>204-011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-014</t>
+          <t>SWI-PRO-MET-204-011</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Carbon Particle Size Distribution and Fines Determination</t>
+          <t>Filter Press Simulation and Cake Filtration Test</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1436,7 +1444,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-014</t>
+          <t>JSEA-PRO-MET-204-011</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1461,7 +1469,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Monthly, and after every regeneration campaign.</t>
+          <t>On each new ore type and whenever plant cake moisture moves.</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
@@ -1487,24 +1495,24 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-014-Carbon-Particle-Size-Distribution-and-Fines-Determination-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-011-Filter-Press-Simulation-and-Cake-Filtration-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>204-015</t>
+          <t>204-012</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-015</t>
+          <t>SWI-PRO-MET-204-012</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Resin Particle Size Distribution and Fines Determination</t>
+          <t>Bond Ball Mill Work Index Test</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1519,7 +1527,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-015</t>
+          <t>JSEA-PRO-MET-204-012</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1544,7 +1552,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Monthly, and after any osmotic shock event or conditioning batch.</t>
+          <t>On each new ore type or ore blend.</t>
         </is>
       </c>
       <c r="L13" s="2" t="n">
@@ -1570,24 +1578,24 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-015-Resin-Particle-Size-Distribution-and-Fines-Determination-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-012-Bond-Ball-Mill-Work-Index-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>204-016</t>
+          <t>204-013</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-016</t>
+          <t>SWI-PRO-MET-204-013</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Dry Sieve Analysis - Ro-Tap RX29 and 200 mm Sieve Set</t>
+          <t>Grind Establishment Test</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1602,7 +1610,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-016</t>
+          <t>JSEA-PRO-MET-204-013</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1627,7 +1635,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>As required by the analysis schedule.</t>
+          <t>On each new ore type, and when a change to the grind target is proposed.</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
@@ -1653,24 +1661,24 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-016-Dry-Sieve-Analysis---Ro-Tap-RX29-and-200-mm-Sieve-Set-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-013-Grind-Establishment-Test-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>204-017</t>
+          <t>204-014</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-017</t>
+          <t>SWI-PRO-MET-204-014</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Sieve Cleaning, Integrity Check and Aperture Verification</t>
+          <t>Carbon Particle Size Distribution and Fines Determination</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1685,7 +1693,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-017</t>
+          <t>JSEA-PRO-MET-204-014</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1710,7 +1718,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>After every use for cleaning; quarterly for integrity and aperture verification.</t>
+          <t>Monthly, and after every regeneration campaign.</t>
         </is>
       </c>
       <c r="L15" s="2" t="n">
@@ -1736,24 +1744,24 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-017-Sieve-Cleaning-Integrity-Check-and-Aperture-Verification-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-014-Carbon-Particle-Size-Distribution-and-Fines-Determination-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>204-018</t>
+          <t>204-015</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-018</t>
+          <t>SWI-PRO-MET-204-015</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Vacuum Filtration of Test Products</t>
+          <t>Resin Particle Size Distribution and Fines Determination</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1768,7 +1776,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-018</t>
+          <t>JSEA-PRO-MET-204-015</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1793,7 +1801,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Every test requiring solid and solution separation.</t>
+          <t>Monthly, and after any osmotic shock event or conditioning batch.</t>
         </is>
       </c>
       <c r="L16" s="2" t="n">
@@ -1819,24 +1827,24 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-018-Vacuum-Filtration-of-Test-Products-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-015-Resin-Particle-Size-Distribution-and-Fines-Determination-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>204-019</t>
+          <t>204-016</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-204-019</t>
+          <t>SWI-PRO-MET-204-016</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Centrifuge Operation for Solution Clarification</t>
+          <t>Dry Sieve Analysis - Ro-Tap RX29 and 200 mm Sieve Set</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1851,7 +1859,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-204-019</t>
+          <t>JSEA-PRO-MET-204-016</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1902,12 +1910,261 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-016-Dry-Sieve-Analysis---Ro-Tap-RX29-and-200-mm-Sieve-Set-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>204-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-017</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Sieve Cleaning, Integrity Check and Aperture Verification</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>204 Met Lab - Physical Testwork</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-204-017</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>After every use for cleaning; quarterly for integrity and aperture verification.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-017-Sieve-Cleaning-Integrity-Check-and-Aperture-Verification-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>204-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-018</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Vacuum Filtration of Test Products</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>204 Met Lab - Physical Testwork</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-204-018</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Every test requiring solid and solution separation.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-204-018-Vacuum-Filtration-of-Test-Products-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>204-019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-019</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Centrifuge Operation for Solution Clarification</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>204 Met Lab - Physical Testwork</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-204-019</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>As required by the analysis schedule.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
           <t>MM-4034-033-OR-03-SWI-PRO-MET-204-019-Centrifuge-Operation-for-Solution-Clarification-RevA.docx</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q17"/>
+  <autoFilter ref="A1:Q20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1918,7 +2175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1928,51 +2185,139 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>No. dokumen</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Jenis</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Isi catatan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>SWI-PRO-MET-204-003</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Particle Size Distribution by Laser Sizer</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the named input arrives: a laser particle size analyser has not been purchased (no laser sizer in ILS quotation Q0023979). The method, frequency and equipment are written when the instrument is resolved.</t>
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-008</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Slurry Viscosity and Rheology Test</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: Steps 3 to 5 follow the Martabe work instructions Measure Viscosity Using Brookfield DV2TLV Viscometer (DOC-3-MET-PMC-WIN-00128-IE) and Measure Viscosity of Slurry Using Marsh Funnel Test (DOC-3-MET-PMC-WIN-00127-IE), v1.0, 25/12/2024. The Martabe method and instruments are adopted. JSEA-PRO-MET-204-008 must be updated for the added hazard before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-008</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Slurry Viscosity and Rheology Test</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) the Marsh funnel source names the ASTM standard funnel but gives no fill volume, no sieving of coarse particles and no result in seconds per quart - set the fill volume and the reporting unit before use; (2) the Brookfield DV2T operating instruction and instrument manual are not received - confirm the spindle range for the plant slurries; (3) set the spindle and speed used for each slurry so all samples are read the same way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-010</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Flocculant Screening and Dose Optimisation Test</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: Steps 4 to 8 are taken from the Martabe work instructions Settling Test with Variance %Strength Flocc (22/03/2025), Effective Treatment Dosage (DOC-3-MET-PMC-WIN-00122-IE) and Flocculant Testwork on Tailing Using Sieve (DOC-3-MET-PMC-WIN-00124-IE), v1.0, 25/12/2024. They are approved for inclusion. Settling cylinders are not purchased; plain 1 L graduated cylinders are approved for use until they are. JSEA-PRO-MET-204-010 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-204-010</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Flocculant Screening and Dose Optimisation Test</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) how the 4 strengths and 4 doses are laid out across the 4 cylinders of a set (Step 4); (2) the basis for 276 g and 12 samples (Step 5); (3) name the Mt. Morgan tailing sample point and the cyanide-bearing return point that replace the Martabe safety carbon screen distributor door and pump PU-372 (see SWI-PRO-MET-201-008); (4) flocculant mixing and ageing time are not stated - Step 2 requires the same ageing for every candidate; (5) bucket size, 10 L or 20 L; (6) the Martabe flocculant make-up SOP is not received; (7) the source reads the settling times as 60, 24 hours, 48 hours - minute 60 is assumed (Step 4); (8) confirm the record folders and forms exist at Mt. Morgan.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1990,49 +2335,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Register seri 204 Physical Testwork (16 dokumen dalam format Heritage).</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Register seri 204 Physical Testwork (19 dokumen dalam format Heritage).</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Data dibaca langsung dari Part 1 dan Part 2 tiap dokumen (judul, tanggal, owner, JSEA ID, area, frekuensi).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Klasifikasi dan padanan Martabe diambil dari docs/Matriks-Rujukan-Martabe.xlsx dan docs/Tabel-SWI-vs-Martabe.xlsx, ditimpa oleh keputusan review bila ada. Format Heritage tidak memuat kolom klasifikasi, jadi klasifikasi hanya ada di register.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Jumlah step dan halaman dihitung dari render dokumen (LibreOffice); halaman bisa sedikit berbeda di Microsoft Word.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Status isi: Final = tanpa tambahan Martabe terbuka; DRAFT FOR REVIEW = ada tambahan Martabe yang menunggu JSEA; Catatan = ada catatan yang perlu ditindaklanjuti.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Sheet "Draft dan open items" memuat paragraf draft, catatan, temuan safety-critical, dan open items di Description of work.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Referensi register: HM-MMM-WHS-REG-XXX-R00-SWI-SWMS, tab SWI-MET.</t>
         </is>

</xml_diff>